<commit_message>
Kop ozgarishlar qoshildi,responsive ham qilindi.
</commit_message>
<xml_diff>
--- a/use/planShablon.xlsx
+++ b/use/planShablon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Front end\Amaliyot\Shablon\use\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E1799F-9956-45A7-9BEE-39E3DF24F810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10216998-F3E0-4CB2-B50B-B4DF61FF1121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2856" yWindow="2184" windowWidth="17280" windowHeight="8964" xr2:uid="{64DD312C-E3FE-4788-AAC3-54FBFBC77CA6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{64DD312C-E3FE-4788-AAC3-54FBFBC77CA6}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t xml:space="preserve">Shablon </t>
   </si>
@@ -48,9 +48,6 @@
     <t>Saytdagi narx</t>
   </si>
   <si>
-    <t>Umumiy %</t>
-  </si>
-  <si>
     <t>Foyda</t>
   </si>
   <si>
@@ -103,6 +100,15 @@
   </si>
   <si>
     <t>Backendchi</t>
+  </si>
+  <si>
+    <t>Kamola</t>
+  </si>
+  <si>
+    <t>Grafik dizayner</t>
+  </si>
+  <si>
+    <t>Foyda uchun qo'yilgan %</t>
   </si>
 </sst>
 </file>
@@ -200,14 +206,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -216,6 +222,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -531,13 +540,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32819456-1F1A-4C36-B598-B85E923E08ED}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.44140625" bestFit="1" customWidth="1"/>
@@ -555,19 +564,19 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -581,7 +590,7 @@
         <f>B2+(B2/100*D2)</f>
         <v>600000</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="8">
         <v>20</v>
       </c>
       <c r="E2" s="2">
@@ -603,7 +612,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2">
         <v>50000</v>
@@ -612,7 +621,7 @@
         <f>B3+(B3/100*D3)</f>
         <v>62500</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="8">
         <v>25</v>
       </c>
       <c r="E3" s="2">
@@ -634,7 +643,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2">
         <v>2000000</v>
@@ -643,7 +652,7 @@
         <f>B4+(B4/100*D4)</f>
         <v>2300000</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="8">
         <v>15</v>
       </c>
       <c r="E4" s="2">
@@ -665,7 +674,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2">
         <v>8000000</v>
@@ -674,7 +683,7 @@
         <f>B5+(B5/100*D5)</f>
         <v>9040000</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="8">
         <v>13</v>
       </c>
       <c r="E5" s="2">
@@ -696,7 +705,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2">
         <v>600000</v>
@@ -705,7 +714,7 @@
         <f>B6+(B6/100*D6)</f>
         <v>690000</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="8">
         <v>15</v>
       </c>
       <c r="E6" s="2">
@@ -727,7 +736,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1">
         <f>SUM(B2:B6)</f>
@@ -756,82 +765,98 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="A9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0.7</v>
+        <v>19</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0.55000000000000004</v>
       </c>
       <c r="D11" s="5">
         <f>H7</f>
         <v>1357400</v>
       </c>
       <c r="E11" s="2">
-        <f>H7*0.7</f>
-        <v>950179.99999999988</v>
+        <f>H7*0.55</f>
+        <v>746570.00000000012</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="4">
-        <v>0.3</v>
+        <v>23</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.15</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="2">
+        <f>H7*0.15</f>
+        <v>203610</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="2">
         <f>H7*0.3</f>
         <v>407220</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="1">
-        <f>SUM(E11:E12)</f>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="1">
+        <f>SUM(E11:E13)</f>
         <v>1357400</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="D11:D14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>